<commit_message>
Added new columns to building template excel + notes
</commit_message>
<xml_diff>
--- a/data_ProjectTemplate/Buildings_ProjectTemplate.xlsx
+++ b/data_ProjectTemplate/Buildings_ProjectTemplate.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AteHe\Desktop\Modellen\LUX_ProjectTemplate\data_ProjectTemplate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bas\Desktop\Github\LUX_ProjectTemplate\data_ProjectTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13149339-643D-44BF-BF53-D5A0B0256AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D5938E-42E7-4EBF-B882-9F02863BABA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{99A50208-934F-4EDD-BF51-6D238E9C57FC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{99A50208-934F-4EDD-BF51-6D238E9C57FC}"/>
   </bookViews>
   <sheets>
     <sheet name="buildings" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">buildings!$A$1:$X$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">buildings!$A$1:$AI$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,9 +43,10 @@
   <authors>
     <author>Ate Hempenius</author>
     <author>Luc Sol</author>
+    <author>Bas Dekker</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{4FF04E4C-5292-4BEB-9F6E-79CE20556081}">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{A901E1C8-ED6F-46C7-9216-F592394CC058}">
       <text>
         <r>
           <rPr>
@@ -70,7 +71,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{57152F91-9E06-4D31-9EEF-EA9B213461F2}">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{C9230EE1-4780-4EFB-B1B6-1BE7358B0103}">
       <text>
         <r>
           <rPr>
@@ -95,7 +96,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="1" shapeId="0" xr:uid="{63B43FE4-2DFE-458F-AA88-0AD3D1781F0B}">
+    <comment ref="C1" authorId="1" shapeId="0" xr:uid="{E0FF640D-8544-41DC-8563-7AE10C206541}">
       <text>
         <r>
           <rPr>
@@ -121,7 +122,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="1" shapeId="0" xr:uid="{3D1D533C-5B41-43B7-9FCE-CE4797AADFC4}">
+    <comment ref="D1" authorId="1" shapeId="0" xr:uid="{E37E7E75-A9C4-44EC-84E5-0DD3201A152C}">
       <text>
         <r>
           <rPr>
@@ -148,7 +149,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="1" shapeId="0" xr:uid="{9DB1F80B-7770-448F-B7C5-B95C6227531F}">
+    <comment ref="E1" authorId="1" shapeId="0" xr:uid="{41C7A490-3074-44E5-B66E-4430C69DA869}">
       <text>
         <r>
           <rPr>
@@ -174,7 +175,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{22E69195-E33A-46EC-B4A6-7699828DF447}">
+    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{6046031E-951E-4ADE-B644-8A2B50DACE2E}">
       <text>
         <r>
           <rPr>
@@ -200,7 +201,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{F1CF16E5-D70A-40ED-8B78-A5BC817F8BCC}">
+    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{51A76FAC-11B5-43FB-A6CF-D8CD32A587C2}">
       <text>
         <r>
           <rPr>
@@ -226,7 +227,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="1" shapeId="0" xr:uid="{1EAEF5C4-DB6F-463A-9305-C54F332EB207}">
+    <comment ref="H1" authorId="1" shapeId="0" xr:uid="{72FB8B4B-699C-4271-A63B-3E2145A89926}">
       <text>
         <r>
           <rPr>
@@ -253,7 +254,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="1" shapeId="0" xr:uid="{5A795051-8748-4EEF-851C-A7F6C88CA63B}">
+    <comment ref="I1" authorId="1" shapeId="0" xr:uid="{4FA6D3F2-A06F-4DC9-BB45-F6ACFB5EB60A}">
       <text>
         <r>
           <rPr>
@@ -279,7 +280,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="1" shapeId="0" xr:uid="{0180DFDE-884B-49DC-AAAB-8EF8231D6AF7}">
+    <comment ref="J1" authorId="1" shapeId="0" xr:uid="{EA94CC62-CD80-4EE1-BD22-89481F4BC4B8}">
       <text>
         <r>
           <rPr>
@@ -304,7 +305,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="1" shapeId="0" xr:uid="{DEB1C7F1-4305-4F7A-A3C4-2A9AFFA49F4B}">
+    <comment ref="K1" authorId="1" shapeId="0" xr:uid="{A5DE0C2C-D045-48F9-8E14-70610C50A960}">
       <text>
         <r>
           <rPr>
@@ -329,7 +330,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="1" shapeId="0" xr:uid="{67A75FA9-0BD1-4CD7-B438-8099B3F91CFD}">
+    <comment ref="L1" authorId="1" shapeId="0" xr:uid="{86668588-C604-4376-BB6F-DDE6E2BA5CBE}">
       <text>
         <r>
           <rPr>
@@ -358,7 +359,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="1" shapeId="0" xr:uid="{A69ACB59-63D9-405D-B1E7-8C5FCD486732}">
+    <comment ref="M1" authorId="1" shapeId="0" xr:uid="{D1F3F318-7009-4066-AF17-1FD682D9E1BE}">
       <text>
         <r>
           <rPr>
@@ -383,7 +384,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="1" shapeId="0" xr:uid="{524DA785-47C5-4088-BB61-39BB2001FD08}">
+    <comment ref="N1" authorId="1" shapeId="0" xr:uid="{201B18FE-F739-4F74-B6EA-177CE892CEAA}">
       <text>
         <r>
           <rPr>
@@ -411,7 +412,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="1" shapeId="0" xr:uid="{C8777648-5A5B-4EBB-828A-593EF2D45AFE}">
+    <comment ref="O1" authorId="1" shapeId="0" xr:uid="{0CD0DD1C-8DB3-4FF6-9A34-E0C838447F8D}">
       <text>
         <r>
           <rPr>
@@ -437,7 +438,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="1" shapeId="0" xr:uid="{819AAD6C-12F9-4998-BED6-422C1A07BFFC}">
+    <comment ref="P1" authorId="1" shapeId="0" xr:uid="{5C0C9415-AD4F-49D3-A28C-F25BFEED0D27}">
       <text>
         <r>
           <rPr>
@@ -463,7 +464,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="1" shapeId="0" xr:uid="{C1656C3D-075F-46BD-BC2F-A2B624759EAD}">
+    <comment ref="Q1" authorId="1" shapeId="0" xr:uid="{59BED9CE-54E9-4B9E-9D84-F748304396B1}">
       <text>
         <r>
           <rPr>
@@ -488,7 +489,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="1" shapeId="0" xr:uid="{313BE7C2-A32D-4855-9081-1060871BCACE}">
+    <comment ref="R1" authorId="1" shapeId="0" xr:uid="{A01A28E4-D4A0-4FE1-88AD-48B8FA949D24}">
       <text>
         <r>
           <rPr>
@@ -513,7 +514,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="1" shapeId="0" xr:uid="{FA84333F-E852-4BA6-ADC3-4C18ED3E848F}">
+    <comment ref="S1" authorId="1" shapeId="0" xr:uid="{491D82B9-B733-485A-A910-EACEFE80BB20}">
       <text>
         <r>
           <rPr>
@@ -538,7 +539,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="1" shapeId="0" xr:uid="{AD24B6AB-1158-43E8-842F-4D714C92F510}">
+    <comment ref="T1" authorId="1" shapeId="0" xr:uid="{6C09CAAC-24AF-4CD7-8117-853FD875811B}">
       <text>
         <r>
           <rPr>
@@ -564,7 +565,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="1" shapeId="0" xr:uid="{6FABADF5-9806-436F-81EC-5A02247424E9}">
+    <comment ref="U1" authorId="1" shapeId="0" xr:uid="{5B3265EF-AECD-417B-8C10-D521EDBC7394}">
       <text>
         <r>
           <rPr>
@@ -590,7 +591,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="1" shapeId="0" xr:uid="{D6946C39-BC7B-45E2-98F8-4E43651FB286}">
+    <comment ref="V1" authorId="1" shapeId="0" xr:uid="{599A232C-ADB8-477D-9E73-8653D09A43F2}">
       <text>
         <r>
           <rPr>
@@ -615,7 +616,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="1" shapeId="0" xr:uid="{EC4AD394-CB46-40F7-891D-56876710C581}">
+    <comment ref="W1" authorId="1" shapeId="0" xr:uid="{0B677F64-7CDF-491F-9A0E-315AA5B9A743}">
       <text>
         <r>
           <rPr>
@@ -639,7 +640,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="1" shapeId="0" xr:uid="{F61542DC-50BE-45B0-BDA5-41015EE1B282}">
+    <comment ref="X1" authorId="1" shapeId="0" xr:uid="{2DB62181-D80B-4A93-98B3-58B901CC97A5}">
       <text>
         <r>
           <rPr>
@@ -662,6 +663,375 @@
 String (mandatory)
 Polygon or MultiPolygon from QGIS
 </t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="2" shapeId="0" xr:uid="{CA31DE9C-0740-4CBE-A618-93CBEEB8BDE2}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">Bas Dekker:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>double</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve"> </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>[Optional]
+Contains the currently installed PV kWp for the address</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="2" shapeId="0" xr:uid="{681F90DA-B9AA-4A97-A0AD-81DAA8867714}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+double [Optional] 
+Contains the maximum potential for installed PV kWp for the address</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="2" shapeId="0" xr:uid="{2BAE4A41-0887-43DD-B837-43C5C7E99BAC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+boolean [optional]
+Has private parking spot at address (TRUE if does not FALSE)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="2" shapeId="0" xr:uid="{A54C0208-C13E-4613-8DB0-90A0B8605716}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+Description of dwelling type</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="2" shapeId="0" xr:uid="{F2A13072-91EE-4FFC-B47D-B08809B9200F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+SBI code</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="2" shapeId="0" xr:uid="{3E1A2E22-F120-4DED-8535-43C147D011A4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+Additional description to the dwelling type
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="2" shapeId="0" xr:uid="{9BD6A832-D922-4A16-A475-AE8EDDB8BFA4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+Type of cooking installation: gasfornuis/inductie
+Not implemented yet</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="2" shapeId="0" xr:uid="{86A2494C-B003-4296-8613-4177D5EBA691}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+Installed type of heating for address
+Not implemented yet</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AG1" authorId="2" shapeId="0" xr:uid="{0D65E3E0-C876-4470-9C2A-D858C61E59B1}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Integer [optional]
+PBL-based
+PBL Dwellingtypes:
+1: vrijstaand
+2: 2-onder-1 kap
+3: rijwoning hoekwoning
+4: rijwoning tussenwoning
+5: appartementen t/m 4 (meergezinswoningen t/m 4 verdiepingen)
+6: appartementen 5&gt;= (meergezinswoningen 5 of meer verdiepingen)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AH1" authorId="2" shapeId="0" xr:uid="{D5635819-3779-4F9C-A7ED-555B036DFEEA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Integer [optional]
+PBL-based
+OwnershipType:
+0: Koop
+1: Particulier Huur
+2: Sociale Huur</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AI1" authorId="2" shapeId="0" xr:uid="{E34DE32E-2D6C-49EE-9924-FCFB27069B95}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+PBL-based
+(Insulation label):
+A+
+A
+B
+C
+D
+E
+F
+G</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AJ1" authorId="2" shapeId="0" xr:uid="{8B25969E-FB90-4FA1-98F3-4E9610C6B31E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+double [optional]
+PBL-based
+Regional climate correction factor: used to compensate for regional climate differences between models for heating consumption</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AK1" authorId="2" shapeId="0" xr:uid="{0AF67813-B71C-4531-9E63-DE4AC391478F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+double [optional]
+PBL-based
+local factor: factor to compensate for local differences between neighbourhoods that affect heating consumption</t>
         </r>
       </text>
     </comment>
@@ -670,7 +1040,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>polygon</t>
   </si>
@@ -742,13 +1112,52 @@
   </si>
   <si>
     <t>gas_consumption_m3pa</t>
+  </si>
+  <si>
+    <t>pv_installed_kwp</t>
+  </si>
+  <si>
+    <t>pv_potential_kwp</t>
+  </si>
+  <si>
+    <t>private_parking</t>
+  </si>
+  <si>
+    <t>house_type</t>
+  </si>
+  <si>
+    <t>sbi_code</t>
+  </si>
+  <si>
+    <t>building_subtype</t>
+  </si>
+  <si>
+    <t>dwelling_type</t>
+  </si>
+  <si>
+    <t>ownership_type</t>
+  </si>
+  <si>
+    <t>insulation_label</t>
+  </si>
+  <si>
+    <t>regional_climate_correction_factor</t>
+  </si>
+  <si>
+    <t>local_factor</t>
+  </si>
+  <si>
+    <t>cooking_type</t>
+  </si>
+  <si>
+    <t>heating_type</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -768,6 +1177,19 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1145,34 +1567,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFCD9D70-6DEB-4390-947E-55D38CEBDCD5}">
-  <dimension ref="A1:X1"/>
-  <sheetFormatPr defaultColWidth="10.1796875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AK1"/>
+  <sheetFormatPr defaultColWidth="10.21875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.81640625" customWidth="1"/>
-    <col min="2" max="2" width="41.54296875" customWidth="1"/>
-    <col min="3" max="3" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.6328125" customWidth="1"/>
-    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="26.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.26953125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="41.08984375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="91.08984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="28.54296875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="22.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="28.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="15" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -1245,9 +1681,47 @@
       <c r="X1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>34</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X1" xr:uid="{CFCD9D70-6DEB-4390-947E-55D38CEBDCD5}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>